<commit_message>
docs: split Layer 0 register and fix all references
- delivery-targets.md       TGT-001..011, sole owner of encode values
- visual-grammar.md         VGR-01..07, ids added to the table
- findings-and-decisions.md RC / DEC / PROP
- competitive-analysis.md   evidence, separated from requirements
- filenames describe content, not layer number, per docs/README.md
- fix stale refs: visual_grammar_requirements.md (x3),
  media-automation-platform-blueprint.html (x1)
- workbook notes now name the owning file per register
</commit_message>
<xml_diff>
--- a/docs/shared/workbooks/design-decisions.xlsx
+++ b/docs/shared/workbooks/design-decisions.xlsx
@@ -554,6 +554,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -724,10 +725,12 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
+    <row r="15"/>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Source of truth: this workbook is a READ-ONLY OVERVIEW. Edit the markdown documents, not these sheets — docs/shared/requirements/ for registers, docs/shared/specs/ for the style contract. Regenerate this file when those change.</t>
+          <t>Source of truth: this workbook is a READ-ONLY OVERVIEW — regenerate it when the documents change. Edit the markdown instead: shared/requirements/delivery-targets.md (TGT), visual-grammar.md (VGR), findings-and-decisions.md (RC/DEC/PROP), competitive-analysis.md (evidence), and shared/specs/style-contract.md (Layer 1).</t>
         </is>
       </c>
     </row>
@@ -1401,6 +1404,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -1725,10 +1729,11 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Source: Lecture_Alive_AI_CompetitiveAnalysis.xlsx, measured via ffprobe / volumedetect. TGT-009 applied identically to all five videos gives cross-video loudness consistency by construction.</t>
+          <t>Owned by docs/shared/requirements/delivery-targets.md — that file is the single source of truth for these values; everything else cites the TGT id rather than repeating the number. Evidence: shared/requirements/competitive-analysis.md. TGT-009 applied identically to all five videos gives cross-video loudness consistency by construction.</t>
         </is>
       </c>
     </row>
@@ -2018,6 +2023,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -2210,10 +2216,11 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>DEC-001 is deferred until Layer 6 — Layer 3 needs only segment-level timing. It is not blocking now, but forced alignment is an unbudgeted component.</t>
+          <t>Owned by docs/shared/requirements/findings-and-decisions.md. DEC-001 is deferred until Layer 6 — Layer 3 needs only segment-level timing. Not blocking now, but forced alignment is an unbudgeted component.</t>
         </is>
       </c>
     </row>

</xml_diff>